<commit_message>
Add a smoothness clarification case and restore profile scenario
</commit_message>
<xml_diff>
--- a/test-cases.xlsx
+++ b/test-cases.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Case Summary" sheetId="1" r:id="R8e833396b8ff4ab8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Steps" sheetId="2" r:id="R3d288b79ada944c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag Guide" sheetId="3" r:id="Rd47fd40afd124ca6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Case Summary" sheetId="1" r:id="Rc7268bb0e27f46d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Steps" sheetId="2" r:id="Rb9f95bd51f6542c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag Guide" sheetId="3" r:id="Rf1a2770afb924c22"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -70,7 +70,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="14">
+  <x:cellXfs count="15">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -99,11 +99,32 @@
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="21">
+  <x:dxfs count="24">
+    <x:dxf>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF9C6500"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
     <x:dxf>
       <x:fill>
         <x:patternFill>
@@ -249,7 +270,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CaseSummaryTable" displayName="CaseSummaryTable" ref="A1:G17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CaseSummaryTable" displayName="CaseSummaryTable" ref="A1:G18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Case ID"/>
     <x:tableColumn id="2" name="Title"/>
@@ -264,7 +285,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="TestStepsTable" displayName="TestStepsTable" ref="A1:C17" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="TestStepsTable" displayName="TestStepsTable" ref="A1:C18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="3">
     <x:tableColumn id="1" name="Case ID"/>
     <x:tableColumn id="2" name="Actions"/>
@@ -653,10 +674,10 @@
         <x:v>MOB-1007</x:v>
       </x:c>
       <x:c r="B9" s="5" t="str">
-        <x:v>Saved profile name is retained in a new session</x:v>
+        <x:v>Saved profile name is retained when the profile is reopened</x:v>
       </x:c>
       <x:c r="C9" s="5" t="str">
-        <x:v>Verify that a saved first and last name remain available in a new session.</x:v>
+        <x:v>Verify that saving a first and last name persists both fields on the same device.</x:v>
       </x:c>
       <x:c r="D9" s="5" t="str">
         <x:v>User is signed in and the Order a ride screen is open.</x:v>
@@ -671,19 +692,19 @@
     </x:row>
     <x:row r="10" ht="72" customHeight="1">
       <x:c r="A10" s="5" t="str">
-        <x:v>MOB-1014</x:v>
+        <x:v>MOB-1010</x:v>
       </x:c>
       <x:c r="B10" s="5" t="str">
-        <x:v>An active ride is restored after signing in on a second device</x:v>
+        <x:v>The side menu opens smoothly</x:v>
       </x:c>
       <x:c r="C10" s="5" t="str">
-        <x:v>Verify that the same account can view its active ride on a second physical phone or emulator.</x:v>
+        <x:v>Verify that opening the side menu produces a smooth visual transition.</x:v>
       </x:c>
       <x:c r="D10" s="5" t="str">
-        <x:v>Device A is a physical Android phone. Device B is a second physical Android phone or an Android emulator. Both devices have the app installed and network access. One test account is available and has no active ride. Both devices are signed out.</x:v>
+        <x:v>User is signed in, the Order a ride screen is open and the side menu is closed.</x:v>
       </x:c>
       <x:c r="E10" s="5" t="str">
-        <x:v>regression, mobile, positive</x:v>
+        <x:v>regression, mobile, usability</x:v>
       </x:c>
       <x:c r="F10" s="5" t="str">
         <x:v>TODO</x:v>
@@ -692,183 +713,196 @@
     </x:row>
     <x:row r="11" ht="72" customHeight="1">
       <x:c r="A11" s="5" t="str">
+        <x:v>MOB-1014</x:v>
+      </x:c>
+      <x:c r="B11" s="5" t="str">
+        <x:v>An active ride is restored after signing in on a second device</x:v>
+      </x:c>
+      <x:c r="C11" s="5" t="str">
+        <x:v>Verify that the same account can view its active ride on a second physical phone or emulator.</x:v>
+      </x:c>
+      <x:c r="D11" s="5" t="str">
+        <x:v>Device A is a physical Android phone. Device B is a second physical Android phone or an Android emulator. Both devices have the app installed and network access. One test account is available and has no active ride. Both devices are signed out.</x:v>
+      </x:c>
+      <x:c r="E11" s="5" t="str">
+        <x:v>regression, mobile, positive</x:v>
+      </x:c>
+      <x:c r="F11" s="5" t="str">
+        <x:v>TODO</x:v>
+      </x:c>
+      <x:c r="G11" s="13"/>
+    </x:row>
+    <x:row r="12" ht="72" customHeight="1">
+      <x:c r="A12" s="5" t="str">
         <x:v>API-2000</x:v>
       </x:c>
-      <x:c r="B11" s="5" t="str">
+      <x:c r="B12" s="5" t="str">
         <x:v>Valid phone and OTP issue a token that authorizes order history</x:v>
       </x:c>
-      <x:c r="C11" s="5" t="str">
+      <x:c r="C12" s="5" t="str">
         <x:v>Verify that a token issued for valid credentials authorizes GET /orders.</x:v>
       </x:c>
-      <x:c r="D11" s="5" t="str">
+      <x:c r="D12" s="5" t="str">
         <x:v>A fresh sandbox session exists.</x:v>
       </x:c>
-      <x:c r="E11" s="5" t="str">
+      <x:c r="E12" s="5" t="str">
         <x:v>smoke, regression, api, authorization, positive</x:v>
       </x:c>
-      <x:c r="F11" s="5" t="str">
+      <x:c r="F12" s="5" t="str">
         <x:v>api-tests/src/test/kotlin/tests/ApiSmokeTest.kt#testValidLoginIssuesWorkingToken</x:v>
       </x:c>
-      <x:c r="G11" s="13" t="str">
+      <x:c r="G12" s="13" t="str">
         <x:v>POST /auth/phone
 POST /auth/otp
 GET /orders</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="72" customHeight="1">
-      <x:c r="A12" s="5" t="str">
+    <x:row r="13" ht="72" customHeight="1">
+      <x:c r="A13" s="5" t="str">
         <x:v>API-2001</x:v>
       </x:c>
-      <x:c r="B12" s="5" t="str">
+      <x:c r="B13" s="5" t="str">
         <x:v>A completed ride becomes the newest order</x:v>
       </x:c>
-      <x:c r="C12" s="5" t="str">
+      <x:c r="C13" s="5" t="str">
         <x:v>Verify that a completed ride becomes the first order in history.</x:v>
       </x:c>
-      <x:c r="D12" s="5" t="str">
+      <x:c r="D13" s="5" t="str">
         <x:v>An authorized session has no active ride; order history contains three orders.</x:v>
       </x:c>
-      <x:c r="E12" s="5" t="str">
+      <x:c r="E13" s="5" t="str">
         <x:v>smoke, regression, api, positive</x:v>
       </x:c>
-      <x:c r="F12" s="5" t="str">
+      <x:c r="F13" s="5" t="str">
         <x:v>api-tests/src/test/kotlin/tests/RideLifecycleApiTest.kt#testCompletedRideAppearsInHistory</x:v>
       </x:c>
-      <x:c r="G12" s="13" t="str">
+      <x:c r="G13" s="13" t="str">
         <x:v>POST /rides
 POST /rides/{id}/complete
 GET /orders</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="72" customHeight="1">
-      <x:c r="A13" s="5" t="str">
+    <x:row r="14" ht="72" customHeight="1">
+      <x:c r="A14" s="5" t="str">
         <x:v>API-2002</x:v>
       </x:c>
-      <x:c r="B13" s="5" t="str">
+      <x:c r="B14" s="5" t="str">
         <x:v>A cancelled ride is not added to order history</x:v>
       </x:c>
-      <x:c r="C13" s="5" t="str">
+      <x:c r="C14" s="5" t="str">
         <x:v>Verify that a cancelled ride is not added to order history.</x:v>
       </x:c>
-      <x:c r="D13" s="5" t="str">
+      <x:c r="D14" s="5" t="str">
         <x:v>An authorized session has no active ride; order history contains three orders.</x:v>
       </x:c>
-      <x:c r="E13" s="5" t="str">
+      <x:c r="E14" s="5" t="str">
         <x:v>regression, api, positive</x:v>
       </x:c>
-      <x:c r="F13" s="5" t="str">
+      <x:c r="F14" s="5" t="str">
         <x:v>api-tests/src/test/kotlin/tests/RideLifecycleApiTest.kt#testCancelledRideDoesNotAppearInHistory</x:v>
       </x:c>
-      <x:c r="G13" s="13" t="str">
+      <x:c r="G14" s="13" t="str">
         <x:v>POST /rides
 POST /rides/{id}/cancel
 GET /orders</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="72" customHeight="1">
-      <x:c r="A14" s="5" t="str">
+    <x:row r="15" ht="72" customHeight="1">
+      <x:c r="A15" s="5" t="str">
         <x:v>API-2003</x:v>
       </x:c>
-      <x:c r="B14" s="5" t="str">
+      <x:c r="B15" s="5" t="str">
         <x:v>Order is rejected without changing history when no driver is available</x:v>
       </x:c>
-      <x:c r="C14" s="5" t="str">
+      <x:c r="C15" s="5" t="str">
         <x:v>Verify that the driver_not_found sandbox state simulates no available driver, rejects ride creation, and leaves order history unchanged.</x:v>
       </x:c>
-      <x:c r="D14" s="5" t="str">
+      <x:c r="D15" s="5" t="str">
         <x:v>An authorized session has no active ride; order history contains three orders.</x:v>
       </x:c>
-      <x:c r="E14" s="5" t="str">
+      <x:c r="E15" s="5" t="str">
         <x:v>regression, api, negative</x:v>
       </x:c>
-      <x:c r="F14" s="5" t="str">
+      <x:c r="F15" s="5" t="str">
         <x:v>api-tests/src/test/kotlin/tests/RideLifecycleApiTest.kt#testDriverNotFoundRejectsOrder</x:v>
       </x:c>
-      <x:c r="G14" s="13" t="str">
+      <x:c r="G15" s="13" t="str">
         <x:v>POST /sandbox/state (setup)
 POST /rides
 GET /orders</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="70" customHeight="1">
-      <x:c r="A15" s="5" t="str">
+    <x:row r="16" ht="70" customHeight="1">
+      <x:c r="A16" s="5" t="str">
         <x:v>API-2004</x:v>
       </x:c>
-      <x:c r="B15" s="5" t="str">
+      <x:c r="B16" s="5" t="str">
         <x:v>Ride options return expected tariffs with prices</x:v>
       </x:c>
-      <x:c r="C15" s="5" t="str">
+      <x:c r="C16" s="5" t="str">
         <x:v>Verify that an authorized ride-options request returns the expected tariff names and prices.</x:v>
       </x:c>
-      <x:c r="D15" s="5" t="str">
+      <x:c r="D16" s="5" t="str">
         <x:v>A valid bearer token is available.</x:v>
       </x:c>
-      <x:c r="E15" s="5" t="str">
+      <x:c r="E16" s="5" t="str">
         <x:v>smoke, regression, api, positive</x:v>
       </x:c>
-      <x:c r="F15" s="5" t="str">
+      <x:c r="F16" s="5" t="str">
         <x:v>api-tests/src/test/kotlin/tests/RideOptionsApiTest.kt#testRideOptionsListTariffsWithPrices</x:v>
       </x:c>
-      <x:c r="G15" s="13" t="str">
+      <x:c r="G16" s="13" t="str">
         <x:v>GET /rides/options</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="84" customHeight="1">
-      <x:c r="A16" s="5" t="str">
+    <x:row r="17" ht="84" customHeight="1">
+      <x:c r="A17" s="5" t="str">
         <x:v>API-2005</x:v>
       </x:c>
-      <x:c r="B16" s="5" t="str">
+      <x:c r="B17" s="5" t="str">
         <x:v>An OTP requested via API is delivered by SMS and authorizes login</x:v>
       </x:c>
-      <x:c r="C16" s="5" t="str">
+      <x:c r="C17" s="5" t="str">
         <x:v>Verify actual SMS delivery through the receiving number's inbox API and authenticate with the received code.</x:v>
       </x:c>
-      <x:c r="D16" s="5" t="str">
+      <x:c r="D17" s="5" t="str">
         <x:v>A valid test number can receive real SMS. Access to the authentication API and the receiving number's SMS inbox API is available. A fresh authentication session exists.</x:v>
       </x:c>
-      <x:c r="E16" s="5" t="str">
+      <x:c r="E17" s="5" t="str">
         <x:v>regression, api, positive</x:v>
       </x:c>
-      <x:c r="F16" s="5" t="str">
+      <x:c r="F17" s="5" t="str">
         <x:v>TODO</x:v>
       </x:c>
-      <x:c r="G16" s="13" t="str">
+      <x:c r="G17" s="13" t="str">
         <x:v>POST /auth/phone
 External SMS inbox API: method and URL must be supplied by the provider.
 POST /auth/otp</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="72" customHeight="1">
-      <x:c r="A17" s="5" t="str">
+    <x:row r="18" ht="72" customHeight="1">
+      <x:c r="A18" s="5" t="str">
         <x:v>API-2007</x:v>
       </x:c>
-      <x:c r="B17" s="5" t="str">
+      <x:c r="B18" s="5" t="str">
         <x:v>An empty destination is rejected without creating an active ride</x:v>
       </x:c>
-      <x:c r="C17" s="5" t="str">
+      <x:c r="C18" s="5" t="str">
         <x:v>Verify that a ride request with an empty destination fails validation and creates no active ride.</x:v>
       </x:c>
-      <x:c r="D17" s="5" t="str">
+      <x:c r="D18" s="5" t="str">
         <x:v>A fresh authorized sandbox session exists with default settings and no active ride.</x:v>
       </x:c>
-      <x:c r="E17" s="5" t="str">
+      <x:c r="E18" s="5" t="str">
         <x:v>regression, api, negative</x:v>
       </x:c>
-      <x:c r="F17" s="5" t="str">
+      <x:c r="F18" s="5" t="str">
         <x:v>TODO</x:v>
       </x:c>
-      <x:c r="G17" s="13" t="str">
+      <x:c r="G18" s="13" t="str">
         <x:v>POST /rides
 GET /rides/active</x:v>
       </x:c>
-    </x:row>
-    <x:row r="18" ht="15" customHeight="1">
-      <x:c r="A18"/>
-      <x:c r="B18"/>
-      <x:c r="C18"/>
-      <x:c r="D18"/>
-      <x:c r="E18"/>
-      <x:c r="F18"/>
     </x:row>
     <x:row r="19" ht="15" customHeight="1">
       <x:c r="A19"/>
@@ -895,19 +929,19 @@
       <x:c r="F21"/>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="A2:G17">
-    <x:cfRule type="expression" dxfId="18" priority="1">
+  <x:conditionalFormatting sqref="A2:G18">
+    <x:cfRule type="expression" dxfId="21" priority="1">
       <x:formula>$F2="TODO"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="F2:F17">
-    <x:cfRule type="expression" dxfId="19" priority="2">
+  <x:conditionalFormatting sqref="F2:F18">
+    <x:cfRule type="expression" dxfId="22" priority="2">
       <x:formula>$F2="TODO"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R060a4f4ee1bf469b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6bd511d15e034eaa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1031,31 +1065,40 @@
       </x:c>
       <x:c r="B9" s="5" t="str">
         <x:v>1. Open the side menu and tap the profile header.
-2. Replace First name with "Anna" and Last name with "Petrova".
-3. Tap Save.
-4. Start a new session.
-5. Open the profile.</x:v>
+2. Replace First name with "Anna" and Last name with "Petrova", then tap Save.
+3. Tap Back, open the side menu and tap the profile header again.</x:v>
       </x:c>
       <x:c r="C9" s="5" t="str">
         <x:v>1. The profile form is displayed.
-2. The fields contain the entered first and last names.
-3. The confirmation "Profile saved" is displayed.
-4. A new session is active.
-5. First name contains "Anna" and Last name contains "Petrova".</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="136" customHeight="1">
+2. The confirmation "Profile saved" is displayed.
+3. First name contains "Anna" and Last name contains "Petrova".</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="60" customHeight="1">
       <x:c r="A10" s="5" t="str">
+        <x:v>MOB-1010</x:v>
+      </x:c>
+      <x:c r="B10" s="5" t="str">
+        <x:v>1. Tap the menu button on the Order a ride screen.
+2. Observe the side menu throughout its opening animation.</x:v>
+      </x:c>
+      <x:c r="C10" s="5" t="str">
+        <x:v>1. The side menu opens.
+2. The menu opens smoothly, without noticeable jerks.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="136" customHeight="1">
+      <x:c r="A11" s="5" t="str">
         <x:v>MOB-1014</x:v>
       </x:c>
-      <x:c r="B10" s="5" t="str">
+      <x:c r="B11" s="5" t="str">
         <x:v>1. Sign in on device A and open Order a ride.
 2. Use pickup "Oak Avenue" and destination "Market Street", select Yellow and tap Order. Record the route, tariff and driver details after a driver is found.
 3. Leave the ride active on device A. Sign in on device B using the same phone number and open Order a ride.
 4. Compare the active ride shown on device B with the ride on device A.
 5. Cancel the ride from device A to clean up.</x:v>
       </x:c>
-      <x:c r="C10" s="5" t="str">
+      <x:c r="C11" s="5" t="str">
         <x:v>1. Device A displays the Order a ride screen.
 2. Device A displays an active ride with a found driver.
 3. Device B restores the existing active ride without placing another order.
@@ -1063,109 +1106,104 @@
 5. Device A confirms cancellation and returns to the ride form.</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="56" customHeight="1">
-      <x:c r="A11" s="5" t="str">
+    <x:row r="12" ht="56" customHeight="1">
+      <x:c r="A12" s="5" t="str">
         <x:v>API-2000</x:v>
       </x:c>
-      <x:c r="B11" s="5" t="str">
+      <x:c r="B12" s="5" t="str">
         <x:v>1. POST /auth/phone with any phone containing at least 8 digits (test data: "+381 64 123 45 67").
 2. POST /auth/otp with the same phone and OTP "1234".
 3. GET /orders with the issued bearer token.</x:v>
       </x:c>
-      <x:c r="C11" s="5" t="str">
+      <x:c r="C12" s="5" t="str">
         <x:v>1. The response is HTTP 200 and the status is "otp_sent".
 2. The response is HTTP 200 and contains a non-empty bearer token.
 3. The response is HTTP 200 and contains the orders collection.</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="80" customHeight="1">
-      <x:c r="A12" s="5" t="str">
+    <x:row r="13" ht="80" customHeight="1">
+      <x:c r="A13" s="5" t="str">
         <x:v>API-2001</x:v>
       </x:c>
-      <x:c r="B12" s="5" t="str">
+      <x:c r="B13" s="5" t="str">
         <x:v>1. POST /rides with any non-empty route and the Yellow tariff (test data: from "Oak Avenue" to "Market Street").
 2. POST /rides/{id}/complete for the created ride.
 3. GET /orders with the bearer token.</x:v>
       </x:c>
-      <x:c r="C12" s="5" t="str">
+      <x:c r="C13" s="5" t="str">
         <x:v>1. The response is HTTP 201; status is "driver_found"; a ride ID and driver details are returned.
 2. The response is HTTP 200; ride status is "completed"; the returned order contains the submitted route and price 2970 euro cents.
 3. The response is HTTP 200; four orders are returned; the first order is the order returned by the completion request.</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="56" customHeight="1">
-      <x:c r="A13" s="5" t="str">
+    <x:row r="14" ht="56" customHeight="1">
+      <x:c r="A14" s="5" t="str">
         <x:v>API-2002</x:v>
       </x:c>
-      <x:c r="B13" s="5" t="str">
+      <x:c r="B14" s="5" t="str">
         <x:v>1. POST /rides with any non-empty route and the Yellow tariff (test data: from "Oak Avenue" to "Market Street").
 2. POST /rides/{id}/cancel for the created ride.
 3. GET /orders with the bearer token.</x:v>
       </x:c>
-      <x:c r="C13" s="5" t="str">
+      <x:c r="C14" s="5" t="str">
         <x:v>1. The response is HTTP 201 and a ride ID is returned.
 2. The response is HTTP 200 and the ride status is "cancelled".
 3. The response is HTTP 200 and the collection exactly matches the three existing orders; no cancelled ride was added.</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="68" customHeight="1">
-      <x:c r="A14" s="5" t="str">
+    <x:row r="15" ht="68" customHeight="1">
+      <x:c r="A15" s="5" t="str">
         <x:v>API-2003</x:v>
       </x:c>
-      <x:c r="B14" s="5" t="str">
+      <x:c r="B15" s="5" t="str">
         <x:v>1. Send POST /sandbox/state with body {"condition":"driver_not_found","enabled":true} to simulate that no driver is available.
 2. POST /rides with any non-empty route and the Yellow tariff (test data: from "Oak Avenue" to "Market Street").
 3. GET /orders with the bearer token.</x:v>
       </x:c>
-      <x:c r="C14" s="5" t="str">
+      <x:c r="C15" s="5" t="str">
         <x:v>1. The response is HTTP 200 and confirms that the state is enabled.
 2. The response is HTTP 409 with the error "No cars found for this route".
 3. The response is HTTP 200 and the collection exactly matches the three existing orders; no rejected ride was added.</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="80" customHeight="1">
-      <x:c r="A15" s="5" t="str">
+    <x:row r="16" ht="80" customHeight="1">
+      <x:c r="A16" s="5" t="str">
         <x:v>API-2004</x:v>
       </x:c>
-      <x:c r="B15" s="5" t="str">
+      <x:c r="B16" s="5" t="str">
         <x:v>1. Send GET /rides/options with a valid bearer token and non-empty from and to query parameters (test data: from "Oak Avenue" to "Market Street").</x:v>
       </x:c>
-      <x:c r="C15" s="5" t="str">
+      <x:c r="C16" s="5" t="str">
         <x:v>1. The response is HTTP 200 and contains exactly these tariff name and price pairs: Yellow — 2970 euro cents, Turquoise — 3454 euro cents, and Minivan — 3905 euro cents; no additional tariffs are returned.</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="106" customHeight="1">
-      <x:c r="A16" s="5" t="str">
+    <x:row r="17" ht="106" customHeight="1">
+      <x:c r="A17" s="5" t="str">
         <x:v>API-2005</x:v>
       </x:c>
-      <x:c r="B16" s="5" t="str">
+      <x:c r="B17" s="5" t="str">
         <x:v>1. Send POST /auth/phone with the test number and record the request time.
 2. Call the receiving number's SMS inbox endpoint (HTTP method and URL must be supplied by the provider). Select a message received after step 1 for this login request and read its code.
 3. Send POST /auth/otp with the same phone number and the received code in the same authentication session.</x:v>
       </x:c>
-      <x:c r="C16" s="5" t="str">
+      <x:c r="C17" s="5" t="str">
         <x:v>1. The response is HTTP 200 with status "otp_sent".
 2. The inbox API returns a newly received SMS addressed to the test number and containing the login code for this request.
 3. The response is HTTP 200 and contains a non-empty bearer token.</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="92" customHeight="1">
-      <x:c r="A17" s="5" t="str">
+    <x:row r="18" ht="92" customHeight="1">
+      <x:c r="A18" s="5" t="str">
         <x:v>API-2007</x:v>
       </x:c>
-      <x:c r="B17" s="5" t="str">
+      <x:c r="B18" s="5" t="str">
         <x:v>1. Send POST /rides with the bearer token and body {"from":"Oak Avenue","to":"","rideOptionId":1}.
 2. Send GET /rides/active with the same token and sandbox session.</x:v>
       </x:c>
-      <x:c r="C17" s="5" t="str">
+      <x:c r="C18" s="5" t="str">
         <x:v>1. The response is HTTP 400 with error "Both from and to are required".
 2. The response is HTTP 404 with error "No active ride".</x:v>
       </x:c>
-    </x:row>
-    <x:row r="18" ht="15" customHeight="1">
-      <x:c r="A18"/>
-      <x:c r="B18"/>
-      <x:c r="C18"/>
     </x:row>
     <x:row r="19" ht="15" customHeight="1">
       <x:c r="A19"/>
@@ -1183,14 +1221,14 @@
       <x:c r="C21"/>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="A2:C17">
-    <x:cfRule type="expression" dxfId="20" priority="1">
-      <x:formula>COUNTIFS('Case Summary'!$A$2:$A$17,$A2,'Case Summary'!$F$2:$F$17,"TODO")&gt;0</x:formula>
+  <x:conditionalFormatting sqref="A2:C18">
+    <x:cfRule type="expression" dxfId="23" priority="1">
+      <x:formula>COUNTIFS('Case Summary'!$A$2:$A$18,$A2,'Case Summary'!$F$2:$F$18,"TODO")&gt;0</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfaf1eaa35ed5421d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R898715ea5fa74cb9"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Register the prepared order-history case as API-2006
</commit_message>
<xml_diff>
--- a/test-cases.xlsx
+++ b/test-cases.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Case Summary" sheetId="1" r:id="Rc7268bb0e27f46d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Steps" sheetId="2" r:id="Rb9f95bd51f6542c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag Guide" sheetId="3" r:id="Rf1a2770afb924c22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Case Summary" sheetId="1" r:id="R017ad822a1a84a1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Steps" sheetId="2" r:id="Rafc3ca8afd044c66"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tag Guide" sheetId="3" r:id="R8a3f9d5c97354eae"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -104,7 +104,27 @@
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="24">
+  <x:dxfs count="27">
+    <x:dxf>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF9C6500"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
     <x:dxf>
       <x:fill>
         <x:patternFill>
@@ -270,7 +290,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CaseSummaryTable" displayName="CaseSummaryTable" ref="A1:G18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CaseSummaryTable" displayName="CaseSummaryTable" ref="A1:G19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="Case ID"/>
     <x:tableColumn id="2" name="Title"/>
@@ -285,7 +305,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="TestStepsTable" displayName="TestStepsTable" ref="A1:C18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="TestStepsTable" displayName="TestStepsTable" ref="A1:C19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="3">
     <x:tableColumn id="1" name="Case ID"/>
     <x:tableColumn id="2" name="Actions"/>
@@ -880,37 +900,52 @@
 POST /auth/otp</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="72" customHeight="1">
+    <x:row r="18" ht="84" customHeight="1">
       <x:c r="A18" s="5" t="str">
+        <x:v>API-2006</x:v>
+      </x:c>
+      <x:c r="B18" s="5" t="str">
+        <x:v>Order history returns the initial order count</x:v>
+      </x:c>
+      <x:c r="C18" s="5" t="str">
+        <x:v>Verify that an authorized order-history request returns HTTP 200 and the initial number of orders.</x:v>
+      </x:c>
+      <x:c r="D18" s="5" t="str">
+        <x:v>A fresh authorized sandbox session exists. Order history contains the three initial orders; no new rides have been completed.</x:v>
+      </x:c>
+      <x:c r="E18" s="5" t="str">
+        <x:v>regression, api, positive</x:v>
+      </x:c>
+      <x:c r="F18" s="5" t="str">
+        <x:v>api-tests/src/test/kotlin/tests/PreparedApiFailureTest.kt#testOrderHistoryReturnsSuccessfulStatus</x:v>
+      </x:c>
+      <x:c r="G18" s="13" t="str">
+        <x:v>GET /orders</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="72" customHeight="1">
+      <x:c r="A19" s="5" t="str">
         <x:v>API-2007</x:v>
       </x:c>
-      <x:c r="B18" s="5" t="str">
+      <x:c r="B19" s="5" t="str">
         <x:v>An empty destination is rejected without creating an active ride</x:v>
       </x:c>
-      <x:c r="C18" s="5" t="str">
+      <x:c r="C19" s="5" t="str">
         <x:v>Verify that a ride request with an empty destination fails validation and creates no active ride.</x:v>
       </x:c>
-      <x:c r="D18" s="5" t="str">
+      <x:c r="D19" s="5" t="str">
         <x:v>A fresh authorized sandbox session exists with default settings and no active ride.</x:v>
       </x:c>
-      <x:c r="E18" s="5" t="str">
+      <x:c r="E19" s="5" t="str">
         <x:v>regression, api, negative</x:v>
       </x:c>
-      <x:c r="F18" s="5" t="str">
+      <x:c r="F19" s="5" t="str">
         <x:v>TODO</x:v>
       </x:c>
-      <x:c r="G18" s="13" t="str">
+      <x:c r="G19" s="13" t="str">
         <x:v>POST /rides
 GET /rides/active</x:v>
       </x:c>
-    </x:row>
-    <x:row r="19" ht="15" customHeight="1">
-      <x:c r="A19"/>
-      <x:c r="B19"/>
-      <x:c r="C19"/>
-      <x:c r="D19"/>
-      <x:c r="E19"/>
-      <x:c r="F19"/>
     </x:row>
     <x:row r="20" ht="15" customHeight="1">
       <x:c r="A20"/>
@@ -929,19 +964,19 @@
       <x:c r="F21"/>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="A2:G18">
-    <x:cfRule type="expression" dxfId="21" priority="1">
+  <x:conditionalFormatting sqref="A2:G19">
+    <x:cfRule type="expression" dxfId="24" priority="1">
       <x:formula>$F2="TODO"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="F2:F18">
-    <x:cfRule type="expression" dxfId="22" priority="2">
+  <x:conditionalFormatting sqref="F2:F19">
+    <x:cfRule type="expression" dxfId="25" priority="2">
       <x:formula>$F2="TODO"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6bd511d15e034eaa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68ec75775b6f4c14"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1192,23 +1227,31 @@
 3. The response is HTTP 200 and contains a non-empty bearer token.</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="92" customHeight="1">
+    <x:row r="18" ht="60" customHeight="1">
       <x:c r="A18" s="5" t="str">
+        <x:v>API-2006</x:v>
+      </x:c>
+      <x:c r="B18" s="5" t="str">
+        <x:v>1. Send GET /orders using the valid bearer token and the same sandbox session.
+2. Inspect the response status and the number of entries in the orders array.</x:v>
+      </x:c>
+      <x:c r="C18" s="5" t="str">
+        <x:v>1. The response status is HTTP 200.
+2. The orders array contains exactly the three initial orders.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="92" customHeight="1">
+      <x:c r="A19" s="5" t="str">
         <x:v>API-2007</x:v>
       </x:c>
-      <x:c r="B18" s="5" t="str">
+      <x:c r="B19" s="5" t="str">
         <x:v>1. Send POST /rides with the bearer token and body {"from":"Oak Avenue","to":"","rideOptionId":1}.
 2. Send GET /rides/active with the same token and sandbox session.</x:v>
       </x:c>
-      <x:c r="C18" s="5" t="str">
+      <x:c r="C19" s="5" t="str">
         <x:v>1. The response is HTTP 400 with error "Both from and to are required".
 2. The response is HTTP 404 with error "No active ride".</x:v>
       </x:c>
-    </x:row>
-    <x:row r="19" ht="15" customHeight="1">
-      <x:c r="A19"/>
-      <x:c r="B19"/>
-      <x:c r="C19"/>
     </x:row>
     <x:row r="20" ht="15" customHeight="1">
       <x:c r="A20"/>
@@ -1221,14 +1264,14 @@
       <x:c r="C21"/>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="A2:C18">
-    <x:cfRule type="expression" dxfId="23" priority="1">
-      <x:formula>COUNTIFS('Case Summary'!$A$2:$A$18,$A2,'Case Summary'!$F$2:$F$18,"TODO")&gt;0</x:formula>
+  <x:conditionalFormatting sqref="A2:C19">
+    <x:cfRule type="expression" dxfId="26" priority="1">
+      <x:formula>COUNTIFS('Case Summary'!$A$2:$A$19,$A2,'Case Summary'!$F$2:$F$19,"TODO")&gt;0</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R898715ea5fa74cb9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R93095dab20e94648"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>